<commit_message>
Expand CEMBI CEEMEA universe to 85 issuers with 4-tab models, regional filtering, and 255 footnotes
</commit_message>
<xml_diff>
--- a/models/ADCB_Credit_Model.xlsx
+++ b/models/ADCB_Credit_Model.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Bank Financials" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital Adequacy &amp; Funding" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Quality Stress Test" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,7 +65,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,19 +75,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001B365D"/>
-        <bgColor rgb="001B365D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F4F8"/>
-        <bgColor rgb="00F2F4F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002C3E50"/>
-        <bgColor rgb="002C3E50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +143,9 @@
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -213,45 +220,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>CEMBI Research</author>
-  </authors>
-  <commentList>
-    <comment ref="B2" authorId="0" shapeId="0">
-      <text>
-        <t>CEMBI CEEMEA Master Research Note
-• [Cognitive Credit / J.P. Morgan] NIM Dynamics &amp; Rate Cycle: Net Interest Margin supported by high proportion of floating-rate commercial loans; fixed-cost customer deposits lag policy rate adjustments.
-• [BRSA / Central Bank Disclosures] Asset Quality &amp; Stage 2 Exposure: NPL ratio remains low with &gt;100% specific coverage. Stage 2 loans closely monitored under macroprudential guidance.
-• Downside Recovery Floor: $76.0 (Base: $100.5)</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>J.P. Morgan</author>
-    <author>Banking Analyst</author>
-  </authors>
-  <commentList>
-    <comment ref="B6" authorId="0" shapeId="0">
-      <text>
-        <t>Net Interest Income driven by loan growth and asset margin repricing.</t>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="1" shapeId="0">
-      <text>
-        <t>Total assets based on audited balance sheets under IFRS 9.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -548,9 +516,9 @@
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -563,7 +531,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CEMBI CEEMEA Financial Institutions Assessment | Country: UAE | Benchmark: ADCBUH 5.05% 2029</t>
+          <t>CEMBI CEEMEA Banking Institution Assessment | Country: UAE (Middle East) | Benchmark: ADCBUH 5.05% 2029</t>
         </is>
       </c>
     </row>
@@ -592,7 +560,7 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Benchmark Senior Paper</t>
+          <t>ADCBUH 5.05% 2029</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -614,12 +582,12 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Loan Product Mix</t>
+          <t>Downside Recovery Floor</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Corporate &amp; Government Entities (54%), Retail Consumer (28%), Treasury &amp; Investments (18%)</t>
+          <t>$76.00</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -629,13 +597,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>NPL: 3.8% (Coverage: 128%)</t>
+          <t>NPL: 3.8% | NIM: 2.8%</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -645,11 +612,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I25"/>
+  <dimension ref="B2:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -669,7 +636,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Historical Audited Statements (2021A - 2024A) and Multi-Year Institutional Projections (2025E - 2027E) | USD Millions</t>
+          <t>Audited Statements (2021A - 2024A) and Multi-Year Projections (2025E - 2027E) | USD Millions</t>
         </is>
       </c>
     </row>
@@ -788,7 +755,7 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Total Operating Income (NII + Fees)</t>
+          <t>Total Operating Income</t>
         </is>
       </c>
       <c r="C9" s="11">
@@ -886,418 +853,661 @@
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Net Loan Impairment Provisions</t>
+          <t>Loan Loss Provisions</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>688.5</v>
+        <v>459</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>650.2</v>
+        <v>433.5</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>726.7</v>
+        <v>484.5</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>765</v>
+        <v>510</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>726.7</v>
+        <v>484.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>688.5</v>
+        <v>459</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>673.2</v>
+        <v>448.8</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Profit Before Tax</t>
-        </is>
-      </c>
-      <c r="C13" s="13">
-        <f>C11-C12</f>
-        <v/>
-      </c>
-      <c r="D13" s="13">
-        <f>D11-D12</f>
-        <v/>
-      </c>
-      <c r="E13" s="13">
-        <f>E11-E12</f>
-        <v/>
-      </c>
-      <c r="F13" s="13">
-        <f>F11-F12</f>
-        <v/>
-      </c>
-      <c r="G13" s="14">
-        <f>G11-G12</f>
-        <v/>
-      </c>
-      <c r="H13" s="14">
-        <f>H11-H12</f>
-        <v/>
-      </c>
-      <c r="I13" s="14">
-        <f>I11-I12</f>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+      <c r="C13" s="11">
+        <f>(C11-C12)*0.80</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>(D11-D12)*0.80</f>
+        <v/>
+      </c>
+      <c r="E13" s="11">
+        <f>(E11-E12)*0.80</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
+        <f>(F11-F12)*0.80</f>
+        <v/>
+      </c>
+      <c r="G13" s="12">
+        <f>(G11-G12)*0.80</f>
+        <v/>
+      </c>
+      <c r="H13" s="12">
+        <f>(H11-H12)*0.80</f>
+        <v/>
+      </c>
+      <c r="I13" s="12">
+        <f>(I11-I12)*0.80</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Net Income / Profit</t>
-        </is>
-      </c>
-      <c r="C14" s="11">
-        <f>C13*0.80</f>
-        <v/>
-      </c>
-      <c r="D14" s="11">
-        <f>D13*0.80</f>
-        <v/>
-      </c>
-      <c r="E14" s="11">
-        <f>E13*0.80</f>
-        <v/>
-      </c>
-      <c r="F14" s="11">
-        <f>F13*0.80</f>
-        <v/>
-      </c>
-      <c r="G14" s="12">
-        <f>G13*0.80</f>
-        <v/>
-      </c>
-      <c r="H14" s="12">
-        <f>H13*0.80</f>
-        <v/>
-      </c>
-      <c r="I14" s="12">
-        <f>I13*0.80</f>
-        <v/>
-      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>II. BALANCE SHEET STRUCTURE (USD M)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>II. BALANCE SHEET STRUCTURE (USD M)</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>120960</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>141120</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>156240</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>168000</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>181440</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>193200</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>204960</v>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Total Assets</t>
+          <t>Gross Customer Loans</t>
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>120960</v>
+        <v>59500</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>141120</v>
+        <v>69700</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>156240</v>
+        <v>78200</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>168000</v>
+        <v>85000</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>181440</v>
+        <v>91800</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>193200</v>
+        <v>98600</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>204960</v>
+        <v>104550</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Gross Customer Loans</t>
+          <t>Customer Deposits</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>59500</v>
+        <v>82880</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>69700</v>
+        <v>95200</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>78200</v>
+        <v>105280</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>85000</v>
+        <v>112000</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>91800</v>
+        <v>119840</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>98600</v>
+        <v>127680</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>104550</v>
+        <v>134400</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Customer Deposits</t>
+          <t>Shareholders' Equity (Tier-1)</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>82880</v>
+        <v>13708.8</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>95200</v>
+        <v>16128</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>105280</v>
+        <v>18144</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>112000</v>
+        <v>20160</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>119840</v>
+        <v>22579.2</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>127680</v>
+        <v>24998.4</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>134400</v>
+        <v>27417.6</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Total Shareholders' Equity (Core Tier-1)</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="n">
-        <v>13708.8</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>16128</v>
-      </c>
-      <c r="E19" s="11" t="n">
-        <v>18144</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>20160</v>
-      </c>
-      <c r="G19" s="12" t="n">
-        <v>22579.2</v>
-      </c>
-      <c r="H19" s="12" t="n">
-        <v>24998.4</v>
-      </c>
-      <c r="I19" s="12" t="n">
-        <v>27417.6</v>
-      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>III. KEY PRUDENTIAL &amp; REGULATORY RATIOS</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>III. PRUDENTIAL &amp; REGULATORY RATIOS (2021A - 2027E)</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="9" t="n"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Net Interest Margin (NIM %)</t>
+        </is>
+      </c>
+      <c r="C20" s="15">
+        <f>C7/C16</f>
+        <v/>
+      </c>
+      <c r="D20" s="15">
+        <f>D7/D16</f>
+        <v/>
+      </c>
+      <c r="E20" s="15">
+        <f>E7/E16</f>
+        <v/>
+      </c>
+      <c r="F20" s="15">
+        <f>F7/F16</f>
+        <v/>
+      </c>
+      <c r="G20" s="16">
+        <f>G7/G16</f>
+        <v/>
+      </c>
+      <c r="H20" s="16">
+        <f>H7/H16</f>
+        <v/>
+      </c>
+      <c r="I20" s="16">
+        <f>I7/I16</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Net Interest Margin (NIM %)</t>
-        </is>
-      </c>
-      <c r="C21" s="15">
-        <f>C7/C17</f>
-        <v/>
-      </c>
-      <c r="D21" s="15">
-        <f>D7/D17</f>
-        <v/>
-      </c>
-      <c r="E21" s="15">
-        <f>E7/E17</f>
-        <v/>
-      </c>
-      <c r="F21" s="15">
-        <f>F7/F17</f>
-        <v/>
-      </c>
-      <c r="G21" s="16">
-        <f>G7/G17</f>
-        <v/>
-      </c>
-      <c r="H21" s="16">
-        <f>H7/H17</f>
-        <v/>
-      </c>
-      <c r="I21" s="16">
-        <f>I7/I17</f>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Cost-to-Income Ratio (CIR %)</t>
+        </is>
+      </c>
+      <c r="C21" s="17">
+        <f>C10/C9</f>
+        <v/>
+      </c>
+      <c r="D21" s="17">
+        <f>D10/D9</f>
+        <v/>
+      </c>
+      <c r="E21" s="17">
+        <f>E10/E9</f>
+        <v/>
+      </c>
+      <c r="F21" s="17">
+        <f>F10/F9</f>
+        <v/>
+      </c>
+      <c r="G21" s="18">
+        <f>G10/G9</f>
+        <v/>
+      </c>
+      <c r="H21" s="18">
+        <f>H10/H9</f>
+        <v/>
+      </c>
+      <c r="I21" s="18">
+        <f>I10/I9</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Cost-to-Income Ratio (CIR %)</t>
-        </is>
-      </c>
-      <c r="C22" s="17">
-        <f>C10/C9</f>
-        <v/>
-      </c>
-      <c r="D22" s="17">
-        <f>D10/D9</f>
-        <v/>
-      </c>
-      <c r="E22" s="17">
-        <f>E10/E9</f>
-        <v/>
-      </c>
-      <c r="F22" s="17">
-        <f>F10/F9</f>
-        <v/>
-      </c>
-      <c r="G22" s="18">
-        <f>G10/G9</f>
-        <v/>
-      </c>
-      <c r="H22" s="18">
-        <f>H10/H9</f>
-        <v/>
-      </c>
-      <c r="I22" s="18">
-        <f>I10/I9</f>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Return on Equity (ROE %)</t>
+        </is>
+      </c>
+      <c r="C22" s="15">
+        <f>C13/C18</f>
+        <v/>
+      </c>
+      <c r="D22" s="15">
+        <f>D13/D18</f>
+        <v/>
+      </c>
+      <c r="E22" s="15">
+        <f>E13/E18</f>
+        <v/>
+      </c>
+      <c r="F22" s="15">
+        <f>F13/F18</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>G13/G18</f>
+        <v/>
+      </c>
+      <c r="H22" s="16">
+        <f>H13/H18</f>
+        <v/>
+      </c>
+      <c r="I22" s="16">
+        <f>I13/I18</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Return on Equity (ROE %)</t>
-        </is>
-      </c>
-      <c r="C23" s="15">
-        <f>C14/C19</f>
-        <v/>
-      </c>
-      <c r="D23" s="15">
-        <f>D14/D19</f>
-        <v/>
-      </c>
-      <c r="E23" s="15">
-        <f>E14/E19</f>
-        <v/>
-      </c>
-      <c r="F23" s="15">
-        <f>F14/F19</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
-        <f>G14/G19</f>
-        <v/>
-      </c>
-      <c r="H23" s="16">
-        <f>H14/H19</f>
-        <v/>
-      </c>
-      <c r="I23" s="16">
-        <f>I14/I19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Return on Assets (ROA %)</t>
-        </is>
-      </c>
-      <c r="C24" s="17">
-        <f>C14/C16</f>
-        <v/>
-      </c>
-      <c r="D24" s="17">
-        <f>D14/D16</f>
-        <v/>
-      </c>
-      <c r="E24" s="17">
-        <f>E14/E16</f>
-        <v/>
-      </c>
-      <c r="F24" s="17">
-        <f>F14/F16</f>
-        <v/>
-      </c>
-      <c r="G24" s="18">
-        <f>G14/G16</f>
-        <v/>
-      </c>
-      <c r="H24" s="18">
-        <f>H14/H16</f>
-        <v/>
-      </c>
-      <c r="I24" s="18">
-        <f>I14/I16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Loan-to-Deposit Ratio (LDR %)</t>
         </is>
       </c>
-      <c r="C25" s="17">
-        <f>C17/C18</f>
-        <v/>
-      </c>
-      <c r="D25" s="17">
-        <f>D17/D18</f>
-        <v/>
-      </c>
-      <c r="E25" s="17">
-        <f>E17/E18</f>
-        <v/>
-      </c>
-      <c r="F25" s="17">
-        <f>F17/F18</f>
-        <v/>
-      </c>
-      <c r="G25" s="18">
-        <f>G17/G18</f>
-        <v/>
-      </c>
-      <c r="H25" s="18">
-        <f>H17/H18</f>
-        <v/>
-      </c>
-      <c r="I25" s="18">
-        <f>I17/I18</f>
+      <c r="C23" s="17">
+        <f>C16/C17</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>D16/D17</f>
+        <v/>
+      </c>
+      <c r="E23" s="17">
+        <f>E16/E17</f>
+        <v/>
+      </c>
+      <c r="F23" s="17">
+        <f>F16/F17</f>
+        <v/>
+      </c>
+      <c r="G23" s="18">
+        <f>G16/G17</f>
+        <v/>
+      </c>
+      <c r="H23" s="18">
+        <f>H16/H17</f>
+        <v/>
+      </c>
+      <c r="I23" s="18">
+        <f>I16/I17</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank — Capital Adequacy &amp; Wholesale Debt Profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory capital tiers, subordinated debt tranches, and liquidity coverage buffers</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>REGULATORY CAPITAL TRANCHE</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>AMOUNT ($M)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>RATIO (%)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>BASEL III MINIMUM</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SURPLUS BUFFER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Common Equity Tier 1 (CET1)</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>17136</v>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>14.2%</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>+0.9% Cushion</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Additional Tier 1 Capital (AT1 Notes)</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>3024</v>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>2.4%</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Tier 2 Subordinated Debt</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>4032</v>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>2.8%</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>2.0%</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>+0.8% Cushion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Total Capital Adequacy Ratio (CAR)</t>
+        </is>
+      </c>
+      <c r="C9" s="10">
+        <f>C6+C7+C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Well Capitalized</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank — Credit Stress &amp; NPL Shock Modeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Stress-testing NPL surges, credit cost shocks (CoR), and capital adequacy depletion</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Prudential Metric</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Base Scenario</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Moderate Macro Shock</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Severe Sovereign / FX Crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>NPL Ratio (%)</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>3.8%</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>4.5%</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>7.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Cost of Risk (bp)</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>60 bp</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>165 bp</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>280 bp</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Annual Provisions ($M)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>510</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>918</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Net Profit Impact ($M)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>1071</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>666.4</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>190.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Post-Stress CAR (%)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>14.1% (Above Minimum)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>